<commit_message>
feat: add posting PDL and Realokasi LITTR modules, adjust table styles globally, and fix request-grant layouts
</commit_message>
<xml_diff>
--- a/table_privileges_mapping.xlsx
+++ b/table_privileges_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\newkotainter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705D2BE5-A504-4DC3-A420-469AC627F36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B123E03-11F3-4C1C-AE87-C9C0499E459A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="117">
   <si>
     <t>NO</t>
   </si>
@@ -325,13 +325,64 @@
   </si>
   <si>
     <t>Tabel login administrator NewKotainter (jika login)</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>Posting PDL</t>
+  </si>
+  <si>
+    <t>BILL52.TRANS_PDL</t>
+  </si>
+  <si>
+    <t>Membaca dan memperbarui status/kolom data transaksi PDL</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>OPHARAPP.OPHAR_TRANS_PDL_LOG</t>
+  </si>
+  <si>
+    <t>Mencatat log perubahan sebelum data PDL diperbarui</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Mencatat riwayat log proses eksekusi Posting PDL</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>bill52.trans_pdl</t>
+  </si>
+  <si>
+    <t>Membaca dan memperbarui status/kolom data transaksi PDL lokal</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>opharapp.ophar_trans_pdl_log</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>CREATE; INSERT</t>
+  </si>
+  <si>
+    <t>Create table ambil dari tabel yang sama di ORACLE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -712,8 +763,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:F42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -723,7 +774,7 @@
     <col min="6" max="6" width="137" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -743,7 +794,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -763,7 +814,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -783,7 +834,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
@@ -803,7 +854,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -823,7 +874,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -843,7 +894,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
@@ -863,7 +914,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>28</v>
       </c>
@@ -883,7 +934,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>31</v>
       </c>
@@ -903,7 +954,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>34</v>
       </c>
@@ -923,7 +974,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>38</v>
       </c>
@@ -943,7 +994,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>42</v>
       </c>
@@ -963,7 +1014,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>45</v>
       </c>
@@ -983,7 +1034,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>48</v>
       </c>
@@ -1003,7 +1054,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>51</v>
       </c>
@@ -1023,7 +1074,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>54</v>
       </c>
@@ -1043,7 +1094,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>56</v>
       </c>
@@ -1063,7 +1114,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>58</v>
       </c>
@@ -1083,7 +1134,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
@@ -1103,7 +1154,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>62</v>
       </c>
@@ -1123,7 +1174,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1143,7 +1194,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>67</v>
       </c>
@@ -1163,7 +1214,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>70</v>
       </c>
@@ -1183,7 +1234,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>73</v>
       </c>
@@ -1203,7 +1254,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>75</v>
       </c>
@@ -1223,7 +1274,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>77</v>
       </c>
@@ -1243,7 +1294,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>79</v>
       </c>
@@ -1263,7 +1314,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>80</v>
       </c>
@@ -1283,7 +1334,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>82</v>
       </c>
@@ -1303,7 +1354,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>84</v>
       </c>
@@ -1323,7 +1374,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>85</v>
       </c>
@@ -1343,7 +1394,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>86</v>
       </c>
@@ -1363,7 +1414,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>87</v>
       </c>
@@ -1383,7 +1434,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>90</v>
       </c>
@@ -1403,7 +1454,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>91</v>
       </c>
@@ -1423,7 +1474,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>96</v>
       </c>
@@ -1441,6 +1492,126 @@
       </c>
       <c r="F36" s="4" t="s">
         <v>99</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>100</v>
+      </c>
+      <c r="B37" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>102</v>
+      </c>
+      <c r="E37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>105</v>
+      </c>
+      <c r="E38" t="s">
+        <v>36</v>
+      </c>
+      <c r="F38" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>107</v>
+      </c>
+      <c r="B39" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" t="s">
+        <v>52</v>
+      </c>
+      <c r="E39" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>109</v>
+      </c>
+      <c r="B40" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" t="s">
+        <v>24</v>
+      </c>
+      <c r="D40" t="s">
+        <v>110</v>
+      </c>
+      <c r="E40" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" t="s">
+        <v>101</v>
+      </c>
+      <c r="C41" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" t="s">
+        <v>113</v>
+      </c>
+      <c r="E41" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>114</v>
+      </c>
+      <c r="B42" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" t="s">
+        <v>24</v>
+      </c>
+      <c r="D42" t="s">
+        <v>35</v>
+      </c>
+      <c r="E42" t="s">
+        <v>36</v>
+      </c>
+      <c r="F42" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>